<commit_message>
Renumber follow-up questions to fund's email order (6.1-6.8, tracker v3)
Steve supplied the fund's original Initial Diligence Questions doc
(archived to inbox/processed), confirming IDs track the fund's own list
order: each request batch = a section, items in the order asked. Old
scattered IDs (2.4-2.7, 4.3, 5.4, 5.5, old 6.1) remapped; safe since
never sent. Working sheet regenerated; ID convention codified in the
tracker header and skill.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wixok8nVACrVF7w1YcZkwZ
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -493,12 +493,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Installment purchase — economics walkthrough</t>
+          <t>Payment-level tape</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -508,31 +508,31 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Walk through the economics of a typical installment purchase, from the swipe through to final payment: revenue lines and their timing (interchange net of network and processor costs, what's charged upfront at origination, what accrues over the term), plus the flow of funds — who pays whom, when, and which entity each flow lands in.</t>
+          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton — revenue lines and timing:] At the swipe, Zed earns interchange on the purchase, net of network and processor costs [Steve: net interchange economics — see 2.7]. At plan opt-in, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for 3/6/12-month terms) is charged to the account. Over the term, add-on interest of 1% of original principal per month is billed on each monthly statement. On early termination, a cancellation fee equal to the current month's interest applies and the upfront fee is retained (both reversed/waived if cancelled in the first month). [Steve: flow of funds — who pays whom, when, and which entity each flow lands in.]</t>
+          <t>To discuss.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Fee mechanics verified against the installment tape (see METHODS.md). The entity/flow-of-funds half cannot be drafted from repo materials — Steve/finance owe it.</t>
+          <t>Positioned as "to discuss" in the 8/5 response — decision owed by Steve on whether to provide raw transaction/payment-level data. A call to scope this was held 2026-08-12 3:30pm Panama time (per email thread); outcome not recorded anywhere in the repo — Steve to say what was agreed so this can move.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Revolver and pay-in-full — economics walkthrough</t>
+          <t>Installment purchase — economics walkthrough</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -542,65 +542,65 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Same walkthrough for a revolving balance and for a pay-in-full statement, to see how the three products differ economically.</t>
+          <t>Walk through the economics of a typical installment purchase, from the swipe through to final payment: revenue lines and their timing (interchange net of network and processor costs, what's charged upfront at origination, what accrues over the term), plus the flow of funds — who pays whom, when, and which entity each flow lands in.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton:] Pay-in-full: Zed earns interchange on spend; no interest or fees if paid by the due date. Revolver: interchange on spend plus interest at 3% per month on the revolving balance; minimum payment per the formula in 1.2. Late fees apply to either on missed payment. [Steve: flow of funds and entity detail, consistent with 2.4.]</t>
+          <t>[draft skeleton — revenue lines and timing:] At the swipe, Zed earns interchange on the purchase, net of network and processor costs [Steve: net interchange economics — see 6.6]. At plan opt-in, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for 3/6/12-month terms) is charged to the account. Over the term, add-on interest of 1% of original principal per month is billed on each monthly statement. On early termination, a cancellation fee equal to the current month's interest applies and the upfront fee is retained (both reversed/waived if cancelled in the first month). [Steve: flow of funds — who pays whom, when, and which entity each flow lands in.]</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as 2.4.</t>
+          <t>Fund email 2026-08-26, item 1. Fee mechanics verified against the installment tape (see METHODS.md). The entity/flow-of-funds half cannot be drafted from repo materials — Steve/finance owe it.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fee schedule confirmation</t>
+          <t>Revolver and pay-in-full — economics walkthrough</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Drafted</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Confirm the fee schedule: add-on rate by tenor, and the origination fee formula (told 0.5% × number of months; 3% on a 6-month term). Is the fee netted from the disbursement or financed into the balance? Refundable on prepayment? Is unearned add-on interest rebated?</t>
+          <t>Same walkthrough for a revolving balance and for a pay-in-full statement, to see how the three products differ economically.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors. There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement. If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
+          <t>[draft skeleton:] Pay-in-full: Zed earns interchange on spend; no interest or fees if paid by the due date. Revolver: interchange on spend plus interest at 3% per month on the revolving balance; minimum payment per the formula in 1.2. Late fees apply to either on missed payment. [Steve: flow of funds and entity detail, consistent with 6.1.]</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
+          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as 6.1.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as % of GMV</t>
+          <t>"Installment fees" field definition</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as a percentage of GMV for the last six months, split domestic vs international if possible.</t>
+          <t>Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -622,53 +622,53 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
+          <t>Fund email 2026-08-26, item 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification pending — see METHODS.md.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Loss figure basis, charge-off policy, restructures</t>
+          <t>Fee schedule confirmation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator? Charge-off policy in DPD, any change since launch, and approach to restructures/re-aging.</t>
+          <t>Confirm the fee schedule: add-on rate by tenor, and the origination fee formula (told 0.5% × number of months; 3% on a 6-month term). Is the fee netted from the disbursement or financed into the balance? Refundable on prepayment? Is unearned add-on interest rebated?</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>[policy half, from 4.1/1.4 as sent:] Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: basis and denominator of the ~2% figure; whether any restructure program exists.]</t>
+          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors. There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement. If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 8. **The ~2% loss figure appears in no repo artifact** — the shared unit econ file implies loan-loss provision ≈ 49% of gross revenue per active account, so ~2% must be a different basis (likely quoted on the 8/12 call or in the deck). Steve must identify where it came from and its intended definition before we answer; getting this wrong contradicts something the fund already heard.</t>
+          <t>Fund email 2026-08-26, item 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Payment-level tape</t>
+          <t>Revenue fields absent from the tape</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -678,31 +678,31 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
+          <t>The tape shows late fees and installment fees but no interchange, annual fee, upfront fee, cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>To discuss.</t>
+          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Positioned as "to discuss" in the 8/5 response — decision owed by Steve on whether to provide raw transaction/payment-level data. A call to scope this was held 2026-08-12 3:30pm Panama time (per email thread); outcome not recorded anywhere in the repo — Steve to say what was agreed so this can move.</t>
+          <t>Fund email 2026-08-26, item 5. Ties to 6.3 — answer both together once the extract's contents are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>"Installment fees" field definition</t>
+          <t>Net interchange as % of GMV</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
+          <t>Net interchange as a percentage of GMV for the last six months, split domestic vs international if possible.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -724,19 +724,19 @@
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification was in progress when this turn paused.</t>
+          <t>Fund email 2026-08-26, item 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Revenue fields absent from the tape</t>
+          <t>BSP rate ceilings and pricing headroom</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -746,31 +746,31 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>The tape shows late fees and installment fees but no interchange, annual fee, upfront fee, cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
+          <t>Both the revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom, and what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
+          <t>[partial draft:] Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. [Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 5. Ties to 5.4 — answer both together once the extract's contents are confirmed.</t>
+          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>BSP rate ceilings and pricing headroom</t>
+          <t>Loss figure basis, charge-off policy, restructures</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -780,19 +780,19 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Both the revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom, and what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
+          <t>What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator? Charge-off policy in DPD, any change since launch, and approach to restructures/re-aging.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. [Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
+          <t>[policy half, from 4.1/1.4 as sent:] Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: basis and denominator of the ~2% figure; whether any restructure program exists.]</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
+          <t>Fund email 2026-08-26, item 8. **The ~2% loss figure appears in no repo artifact** — the shared unit econ file implies loan-loss provision ≈ 49% of gross revenue per active account, so ~2% must be a different basis (likely quoted on the 8/12 call or in the deck). Steve must identify where it came from and its intended definition before we answer; getting this wrong contradicts something the fund already heard.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close 5.1 per Steve; 8/26 batch keeps the email's own numbers 1-8 (v4)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wixok8nVACrVF7w1YcZkwZ
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -493,12 +493,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Payment-level tape</t>
+          <t>Installment purchase — economics walkthrough</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -508,31 +508,31 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
+          <t>Walk through the economics of a typical installment purchase, from the swipe through to final payment: revenue lines and their timing (interchange net of network and processor costs, what's charged upfront at origination, what accrues over the term), plus the flow of funds — who pays whom, when, and which entity each flow lands in.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>To discuss.</t>
+          <t>[draft skeleton — revenue lines and timing:] At the swipe, Zed earns interchange on the purchase, net of network and processor costs [Steve: net interchange economics — see item 6]. At plan opt-in, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for 3/6/12-month terms) is charged to the account. Over the term, add-on interest of 1% of original principal per month is billed on each monthly statement. On early termination, a cancellation fee equal to the current month's interest applies and the upfront fee is retained (both reversed/waived if cancelled in the first month). [Steve: flow of funds — who pays whom, when, and which entity each flow lands in.]</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Positioned as "to discuss" in the 8/5 response — decision owed by Steve on whether to provide raw transaction/payment-level data. A call to scope this was held 2026-08-12 3:30pm Panama time (per email thread); outcome not recorded anywhere in the repo — Steve to say what was agreed so this can move.</t>
+          <t>Fund email 2026-08-26, item 1. Fee mechanics verified against the installment tape (see METHODS.md). The entity/flow-of-funds half cannot be drafted from repo materials — Steve/finance owe it.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Installment purchase — economics walkthrough</t>
+          <t>Revolver and pay-in-full — economics walkthrough</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -542,31 +542,31 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Walk through the economics of a typical installment purchase, from the swipe through to final payment: revenue lines and their timing (interchange net of network and processor costs, what's charged upfront at origination, what accrues over the term), plus the flow of funds — who pays whom, when, and which entity each flow lands in.</t>
+          <t>Same walkthrough for a revolving balance and for a pay-in-full statement, to see how the three products differ economically.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton — revenue lines and timing:] At the swipe, Zed earns interchange on the purchase, net of network and processor costs [Steve: net interchange economics — see 6.6]. At plan opt-in, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for 3/6/12-month terms) is charged to the account. Over the term, add-on interest of 1% of original principal per month is billed on each monthly statement. On early termination, a cancellation fee equal to the current month's interest applies and the upfront fee is retained (both reversed/waived if cancelled in the first month). [Steve: flow of funds — who pays whom, when, and which entity each flow lands in.]</t>
+          <t>[draft skeleton:] Pay-in-full: Zed earns interchange on spend; no interest or fees if paid by the due date. Revolver: interchange on spend plus interest at 3% per month on the revolving balance; minimum payment per the formula in 1.2. Late fees apply to either on missed payment. [Steve: flow of funds and entity detail, consistent with item 1.]</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Fee mechanics verified against the installment tape (see METHODS.md). The entity/flow-of-funds half cannot be drafted from repo materials — Steve/finance owe it.</t>
+          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Revolver and pay-in-full — economics walkthrough</t>
+          <t>"Installment fees" field definition</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -576,99 +576,99 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Same walkthrough for a revolving balance and for a pay-in-full statement, to see how the three products differ economically.</t>
+          <t>Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton:] Pay-in-full: Zed earns interchange on spend; no interest or fees if paid by the due date. Revolver: interchange on spend plus interest at 3% per month on the revolving balance; minimum payment per the formula in 1.2. Late fees apply to either on missed payment. [Steve: flow of funds and entity detail, consistent with 6.1.]</t>
+          <t>To be provided.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as 6.1.</t>
+          <t>Fund email 2026-08-26, item 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification pending — see METHODS.md.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>"Installment fees" field definition</t>
+          <t>Fee schedule confirmation</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
+          <t>Confirm the fee schedule: add-on rate by tenor, and the origination fee formula (told 0.5% × number of months; 3% on a 6-month term). Is the fee netted from the disbursement or financed into the balance? Refundable on prepayment? Is unearned add-on interest rebated?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>To be provided.</t>
+          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors. There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement. If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification pending — see METHODS.md.</t>
+          <t>Fund email 2026-08-26, item 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fee schedule confirmation</t>
+          <t>Revenue fields absent from the tape</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Drafted</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Confirm the fee schedule: add-on rate by tenor, and the origination fee formula (told 0.5% × number of months; 3% on a 6-month term). Is the fee netted from the disbursement or financed into the balance? Refundable on prepayment? Is unearned add-on interest rebated?</t>
+          <t>The tape shows late fees and installment fees but no interchange, annual fee, upfront fee, cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors. There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement. If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
+          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
+          <t>Fund email 2026-08-26, item 5. Ties to item 3 — answer both together once the extract's contents are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Revenue fields absent from the tape</t>
+          <t>Net interchange as % of GMV</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -678,31 +678,31 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>The tape shows late fees and installment fees but no interchange, annual fee, upfront fee, cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
+          <t>Net interchange as a percentage of GMV for the last six months, split domestic vs international if possible.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
+          <t>To be provided.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 5. Ties to 6.3 — answer both together once the extract's contents are confirmed.</t>
+          <t>Fund email 2026-08-26, item 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as % of GMV</t>
+          <t>BSP rate ceilings and pricing headroom</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -712,31 +712,31 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as a percentage of GMV for the last six months, split domestic vs international if possible.</t>
+          <t>Both the revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom, and what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>To be provided.</t>
+          <t>[partial draft:] Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. [Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
+          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>BSP rate ceilings and pricing headroom</t>
+          <t>Loss figure basis, charge-off policy, restructures</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -746,59 +746,25 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Both the revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom, and what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
+          <t>What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator? Charge-off policy in DPD, any change since launch, and approach to restructures/re-aging.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. [Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
+          <t>[policy half, from 4.1/1.4 as sent:] Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: basis and denominator of the ~2% figure; whether any restructure program exists.]</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Loss figure basis, charge-off policy, restructures</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator? Charge-off policy in DPD, any change since launch, and approach to restructures/re-aging.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>[policy half, from 4.1/1.4 as sent:] Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: basis and denominator of the ~2% figure; whether any restructure program exists.]</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
           <t>Fund email 2026-08-26, item 8. **The ~2% loss figure appears in no repo artifact** — the shared unit econ file implies loan-loss provision ≈ 49% of gross revenue per active account, so ~2% must be a different basis (likely quoted on the 8/12 call or in the deck). Steve must identify where it came from and its intended definition before we answer; getting this wrong contradicts something the fund already heard.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Claude: revise (see notes),Discuss"</formula1>
     </dataValidation>
   </dataValidations>
@@ -812,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1154,52 +1120,79 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Installment plan tape</t>
+          <t>Payment-level tape</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Per installment plan: plan ID, origination date, term, fee, status, cancellation/acceleration date and reason.</t>
+          <t>Per transaction/payment: full payment-level tape (charge date, payment date, amount) for all accounts since inception — transactions and payments, not statement summaries.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Provided — plan-level installment tape (plan ID, opt-in date, tenure, upfront fee, monthly interest, status by month, termination date/source), also in Data Room / Loan Tape.</t>
+          <t>To discuss.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>email 2026-08-21 ("close out the last open item on our side (5.2)"); `Installment Tape_20260814.xlsx` in Data Room / Loan Tape</t>
+          <t>"To discuss" sent in the 8/5 response sheet; scoped on the 2026-08-12 call and since resolved</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Installment plan tape</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Per installment plan: plan ID, origination date, term, fee, status, cancellation/acceleration date and reason.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Provided — plan-level installment tape (plan ID, opt-in date, tenure, upfront fee, monthly interest, status by month, termination date/source), also in Data Room / Loan Tape.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>email 2026-08-21 ("close out the last open item on our side (5.2)"); `Installment Tape_20260814.xlsx` in Data Room / Loan Tape</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Cohort performance file</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Per cohort: monthly origination, outstanding, and cumulative gross/net loss by MOB, split purchase vs. installment.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>The loan tape shows unique cardholders and their origination cohort, which can be joined with the statement tape to show, by unique cardholder, statement charges and credits. We added gross installment conversions as well. DPD columns show what statements balances ever went past due or are currently past due. The statement data can be used to reconstruct every unique cardholders charges and payment history by using the UID key.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>response sheet 2026-08-05</t>
         </is>

</xml_diff>

<commit_message>
Process 8/12 call notes (Granola): 5.1 resolution + ~2% loss basis (v5)
Call notes downloaded from Granola share link into inbox, propagated,
archived to processed. 5.1: Raymond doesn't want a transaction dump; the
statement tape covers the intent. Item 8's ~2% figure grounded: dollars
originated that go past due, 1-3% target, per the call — draft upgraded,
exact computation still to verify in BQ. Context notes on items 2 and 7.
README gains a who-owes-what table: Raymond owes indicative terms.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wixok8nVACrVF7w1YcZkwZ
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -554,7 +554,7 @@
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1.</t>
+          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1. Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
+          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md); on the 8/12 call we already told them "all at regulatory maximums" (3%/mo ≈ 36.5% APR), so "confirmed" is consistent. The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
         </is>
       </c>
     </row>
@@ -751,14 +751,14 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>[policy half, from 4.1/1.4 as sent:] Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: basis and denominator of the ~2% figure; whether any restructure program exists.]</t>
+          <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume — not an annualized NCL rate. We manage to a 1–3% target range and are currently at ~2%, in line with US prime credit card benchmarks. [Steve/Claude: confirm the exact DPD threshold and computation against the warehouse before sending.] On policy: per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: whether any restructure program exists.]</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 8. **The ~2% loss figure appears in no repo artifact** — the shared unit econ file implies loan-loss provision ≈ 49% of gross revenue per active account, so ~2% must be a different basis (likely quoted on the 8/12 call or in the deck). Steve must identify where it came from and its intended definition before we answer; getting this wrong contradicts something the fund already heard.</t>
+          <t>Fund email 2026-08-26, item 8. Basis grounded in the 8/12 call notes ("dollars originated that go past due; target 1–3%, currently ~2%, in line with US prime benchmarks") — the fund heard this live, so the written answer must match it. The exact computation (DPD threshold, as-of date, cumulative vs cohort) is not specified in the notes; verify in BigQuery and record in METHODS.md before approving. Distinct from the unit econ provision line (~49% of gross revenue per active account) — if the fund juxtaposes the two, the reconciliation is originated-volume denominator vs revenue denominator.</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>"To discuss" sent in the 8/5 response sheet; scoped on the 2026-08-12 call and since resolved</t>
+          <t>"To discuss" sent in the 8/5 response sheet; resolved on the 2026-08-12 call</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync working sheet: Steve's item 1 walkthrough, item 2 templated from it (v6)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wixok8nVACrVF7w1YcZkwZ
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -513,14 +513,18 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton — revenue lines and timing:] At the swipe, Zed earns interchange on the purchase, net of network and processor costs [Steve: net interchange economics — see item 6]. At plan opt-in, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for 3/6/12-month terms) is charged to the account. Over the term, add-on interest of 1% of original principal per month is billed on each monthly statement. On early termination, a cancellation fee equal to the current month's interest applies and the upfront fee is retained (both reversed/waived if cancelled in the first month). [Steve: flow of funds — who pays whom, when, and which entity each flow lands in.]</t>
+          <t>Interchange: at the swipe, Zed earns interchange on an installment-enrolled purchase exactly as on any other transaction (net interchange economics covered in item 6).
+Origination: at enrollment, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
+Over the term: add-on interest of 1% × original principal is billed on each monthly statement — so by end of term, total interest of 3% / 6% / 12% of principal has been charged for the 3 / 6 / 12-month terms.
+Early termination: a cancellation fee equal to the current statement cycle's interest is charged and the upfront fee is retained, with one exception — if a purchase is enrolled into installments and cancelled within that same first statement cycle, we charge no interest and reverse the upfront fee. Nothing has been billed at that point and the user hasn't yet floated any of the purchase via installments, so we treat it as a foot fault and allow them to unwind the enrollment without any implications.
+[Steve: the question also asks for the flow of funds — who pays whom, when, and which entity each flow lands in. Answer here, or handle on the follow-up call?]</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Fee mechanics verified against the installment tape (see METHODS.md). The entity/flow-of-funds half cannot be drafted from repo materials — Steve/finance owe it.</t>
+          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet sync 2026-09-01), lightly restructured per his note; fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds/entity half still unanswered — kept as an explicit placeholder.</t>
         </is>
       </c>
     </row>
@@ -537,7 +541,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -547,7 +551,11 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>[draft skeleton:] Pay-in-full: Zed earns interchange on spend; no interest or fees if paid by the due date. Revolver: interchange on spend plus interest at 3% per month on the revolving balance; minimum payment per the formula in 1.2. Late fees apply to either on missed payment. [Steve: flow of funds and entity detail, consistent with item 1.]</t>
+          <t>Interchange: identical to the installment case — at the swipe, Zed earns interchange on the purchase like any other transaction, regardless of how the balance is later paid.
+Pay-in-full: charges aggregate into the statement balance at cycle end. If the cardholder pays the statement balance in full by the due date, no interest or fees are ever charged — the economics to Zed are interchange only.
+Revolving: if the cardholder pays at least the minimum payment (formula per our response to 1.2) but less than the full statement balance, the unpaid remainder revolves and accrues interest at 3% per month. Only charges made after the revolving launch are eligible to revolve.
+Missed payment: if the minimum payment is not met by the due date, late fees are charged, the account becomes past due, and a hard card freeze applies at DPD 1 (per our response to 1.4).
+[Steve: flow of funds and entity detail, same as item 1.]</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix item 1: installment enrollment is post-purchase, not at swipe (v7)
Per Steve: feature works like AmEx Pay Over Time — purchases are made
plain, become enrollment-eligible only for their statement cycle, and the
installment economics apply only upon enrollment. Item 2 opener aligned.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wixok8nVACrVF7w1YcZkwZ
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -513,8 +513,8 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Interchange: at the swipe, Zed earns interchange on an installment-enrolled purchase exactly as on any other transaction (net interchange economics covered in item 6).
-Origination: at enrollment, an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
+          <t>At the swipe, there is no installment dimension yet: the user simply makes a purchase, and Zed earns interchange on it like any other transaction (net interchange economics covered in item 6). Our installment feature works much like AmEx's "Pay Over Time": after the purchase, certain transactions are eligible for installment enrollment, and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
+Origination: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
 Over the term: add-on interest of 1% × original principal is billed on each monthly statement — so by end of term, total interest of 3% / 6% / 12% of principal has been charged for the 3 / 6 / 12-month terms.
 Early termination: a cancellation fee equal to the current statement cycle's interest is charged and the upfront fee is retained, with one exception — if a purchase is enrolled into installments and cancelled within that same first statement cycle, we charge no interest and reverse the upfront fee. Nothing has been billed at that point and the user hasn't yet floated any of the purchase via installments, so we treat it as a foot fault and allow them to unwind the enrollment without any implications.
 [Steve: the question also asks for the flow of funds — who pays whom, when, and which entity each flow lands in. Answer here, or handle on the follow-up call?]</t>
@@ -524,7 +524,7 @@
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet sync 2026-09-01), lightly restructured per his note; fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds/entity half still unanswered — kept as an explicit placeholder.</t>
+          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet sync 2026-09-01), restructured per his note and corrected per his follow-up: enrollment is post-purchase (AmEx Pay-Over-Time-style) — at swipe there is no installment attribute, and eligibility lasts only for the purchase's statement cycle. Fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds/entity half still unanswered — kept as an explicit placeholder.</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Interchange: identical to the installment case — at the swipe, Zed earns interchange on the purchase like any other transaction, regardless of how the balance is later paid.
+          <t>Interchange: as in item 1, every purchase earns Zed interchange at the swipe — payment behavior (pay in full, revolve, or installment enrollment) plays out afterwards and never changes the transaction-level economics.
 Pay-in-full: charges aggregate into the statement balance at cycle end. If the cardholder pays the statement balance in full by the due date, no interest or fees are ever charged — the economics to Zed are interchange only.
 Revolving: if the cardholder pays at least the minimum payment (formula per our response to 1.2) but less than the full statement balance, the unpaid remainder revolves and accrues interest at 3% per month. Only charges made after the revolving launch are eligible to revolve.
 Missed payment: if the minimum payment is not met by the due date, late fees are charged, the account becomes past due, and a hard card freeze applies at DPD 1 (per our response to 1.4).

</xml_diff>

<commit_message>
Funds flow diagram → Data Room/Product; items 1-2 placeholders resolved (v8)
- Built Installment Funds Flow_20260902.pdf collaboratively with Steve (four-party
  purchase flow, Part 2 customer-Zed installment billing, MPD rule)
- Steve confirmed: first 1/X bills in enrollment cycle with the fee; monthly billing
  = 1/X + 1% add-on; single entity, settlement funded from Zed's own balance sheet
- Synced Steve's item 1 wording edits from working sheet; regenerated sheet
- METHODS.md entry for the diagram; SHARED-LOG row deferred until Box upload

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -513,18 +513,18 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>At the swipe, there is no installment dimension yet: the user simply makes a purchase, and Zed earns interchange on it like any other transaction (net interchange economics covered in item 6). Our installment feature works much like AmEx's "Pay Over Time": after the purchase, certain transactions are eligible for installment enrollment, and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
-Origination: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
+          <t>At the swipe, there is no installment dimension yet: the user simply makes a purchase, and Zed earns interchange on it like any other transaction (net interchange economics covered in item 6). Our installment feature works much like AmEx's "Pay Over Time": after the purchase, certain transactions are eligible for installment enrollment and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
+Upon enrollment: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
 Over the term: add-on interest of 1% × original principal is billed on each monthly statement — so by end of term, total interest of 3% / 6% / 12% of principal has been charged for the 3 / 6 / 12-month terms.
 Early termination: a cancellation fee equal to the current statement cycle's interest is charged and the upfront fee is retained, with one exception — if a purchase is enrolled into installments and cancelled within that same first statement cycle, we charge no interest and reverse the upfront fee. Nothing has been billed at that point and the user hasn't yet floated any of the purchase via installments, so we treat it as a foot fault and allow them to unwind the enrollment without any implications.
-[Steve: the question also asks for the flow of funds — who pays whom, when, and which entity each flow lands in. Answer here, or handle on the follow-up call?]</t>
+Flow of funds: see the Installment Funds Flow diagram in Data Room / Product. In short: at purchase, Zed funds the merchant T+1 through Mastercard from its own balance sheet (we have no bank funding partner) and earns interchange; every flow after that is between the customer and Zed — the upfront fee and the first 1/X billing land on the enrollment-cycle statement, and each statement's installment billing converts back to revolving balance and must be paid in full by that cycle's due date under our Minimum Payment Due rules.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet sync 2026-09-01), restructured per his note and corrected per his follow-up: enrollment is post-purchase (AmEx Pay-Over-Time-style) — at swipe there is no installment attribute, and eligibility lasts only for the purchase's statement cycle. Fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds/entity half still unanswered — kept as an explicit placeholder.</t>
+          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet syncs 2026-09-01/02), restructured per his notes: enrollment is post-purchase (AmEx Pay-Over-Time-style) — at swipe there is no installment attribute, and eligibility lasts only for the purchase's statement cycle. Fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds placeholder resolved 2026-09-02 by the diagram (built collaboratively with Steve; his confirmations: first 1/X bills in the enrollment cycle alongside the fee; monthly billing = 1/X + 1% add-on; single-entity issuer funded off Zed's own balance sheet, no bank partner; acquirer collapsed into the network rail; early termination as footnote only). PDF not yet uploaded to Box — SHARED-LOG row waits for Steve's confirmation.</t>
         </is>
       </c>
     </row>
@@ -555,14 +555,14 @@
 Pay-in-full: charges aggregate into the statement balance at cycle end. If the cardholder pays the statement balance in full by the due date, no interest or fees are ever charged — the economics to Zed are interchange only.
 Revolving: if the cardholder pays at least the minimum payment (formula per our response to 1.2) but less than the full statement balance, the unpaid remainder revolves and accrues interest at 3% per month. Only charges made after the revolving launch are eligible to revolve.
 Missed payment: if the minimum payment is not met by the due date, late fees are charged, the account becomes past due, and a hard card freeze applies at DPD 1 (per our response to 1.4).
-[Steve: flow of funds and entity detail, same as item 1.]</t>
+Flow of funds: the purchase-side flow (merchant settlement, interchange, Zed funding from its own balance sheet) is identical for all three behaviors — see the Installment Funds Flow diagram in Data Room / Product, Part 1. For revolvers and pay-in-full, everything after settlement is simply the customer paying Zed against the monthly statement.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 2. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1. Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
+          <t>Fund email 2026-08-26, item 2. Flow-of-funds placeholder resolved 2026-09-02 via the same diagram as item 1. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1. Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renumber 8/26 batch: bullets 1-8 -> items 6-13, verbatim questions (v9)
- Continues the tracker's running numbering per Steve (avoids collision with
  references to prior items like 1.2); multi-part bullets split .1/.2/.3
- 6.1/6.2, 9.1-9.3, 12.1/12.2, 13.1-13.3; splits carry independent statuses
- Questions quoted verbatim from Raymond's email, email bullet numbers kept
- Skill ID convention updated; working sheet regenerated (14 open/drafted rows)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -508,243 +508,242 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Walk through the economics of a typical installment purchase, from the swipe through to final payment: revenue lines and their timing (interchange net of network and processor costs, what's charged upfront at origination, what accrues over the term), plus the flow of funds — who pays whom, when, and which entity each flow lands in.</t>
+          <t>1. Could you walk us through the economics of a typical installment purchase, from the swipe through to final payment? We're mainly after the revenue lines and their timing: what you earn on the transaction itself (interchange, net of network and processor costs), what's charged upfront at origination, and what accrues over the term.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>At the swipe, there is no installment dimension yet: the user simply makes a purchase, and Zed earns interchange on it like any other transaction (net interchange economics covered in item 6). Our installment feature works much like AmEx's "Pay Over Time": after the purchase, certain transactions are eligible for installment enrollment and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
+          <t>At the swipe, there is no installment dimension yet: the user simply makes a purchase, and Zed earns interchange on it like any other transaction (net interchange economics covered in 11). Our installment feature works much like AmEx's "Pay Over Time": after the purchase, certain transactions are eligible for installment enrollment and a purchase is only eligible during the statement cycle in which it was made. If the user enrolls an eligible purchase into installments, the dynamics below follow.
 Upon enrollment: an upfront fee of 0.5% × term months (1.5% / 3% / 6% for the 3 / 6 / 12-month terms, respectively) is charged to the account and billed in its entirety in the statement cycle in which the purchase was enrolled.
 Over the term: add-on interest of 1% × original principal is billed on each monthly statement — so by end of term, total interest of 3% / 6% / 12% of principal has been charged for the 3 / 6 / 12-month terms.
-Early termination: a cancellation fee equal to the current statement cycle's interest is charged and the upfront fee is retained, with one exception — if a purchase is enrolled into installments and cancelled within that same first statement cycle, we charge no interest and reverse the upfront fee. Nothing has been billed at that point and the user hasn't yet floated any of the purchase via installments, so we treat it as a foot fault and allow them to unwind the enrollment without any implications.
-Flow of funds: see the Installment Funds Flow diagram in Data Room / Product. In short: at purchase, Zed funds the merchant T+1 through Mastercard from its own balance sheet (we have no bank funding partner) and earns interchange; every flow after that is between the customer and Zed — the upfront fee and the first 1/X billing land on the enrollment-cycle statement, and each statement's installment billing converts back to revolving balance and must be paid in full by that cycle's due date under our Minimum Payment Due rules.</t>
+Early termination: a cancellation fee equal to the current statement cycle's interest is charged and the upfront fee is retained, with one exception — if a purchase is enrolled into installments and cancelled within that same first statement cycle, we charge no interest and reverse the upfront fee. Nothing has been billed at that point and the user hasn't yet floated any of the purchase via installments, so we treat it as a foot fault and allow them to unwind the enrollment without any implications.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 1. Steve's own explanation (working-sheet syncs 2026-09-01/02), restructured per his notes: enrollment is post-purchase (AmEx Pay-Over-Time-style) — at swipe there is no installment attribute, and eligibility lasts only for the purchase's statement cycle. Fee mechanics verified against the installment tape (see METHODS.md). Flow-of-funds placeholder resolved 2026-09-02 by the diagram (built collaboratively with Steve; his confirmations: first 1/X bills in the enrollment cycle alongside the fee; monthly billing = 1/X + 1% add-on; single-entity issuer funded off Zed's own balance sheet, no bank partner; acquirer collapsed into the network rail; early termination as footnote only). PDF not yet uploaded to Box — SHARED-LOG row waits for Steve's confirmation.</t>
+          <t>Fund email 2026-08-26, bullet 1 (economics half; flow of funds split to 6.2). Steve's own explanation (working-sheet syncs 2026-09-01/02), restructured per his notes: enrollment is post-purchase (AmEx Pay-Over-Time-style) — at swipe there is no installment attribute, and eligibility lasts only for the purchase's statement cycle. Fee mechanics verified against the installment tape (see METHODS.md).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Installment purchase — flow of funds</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1 (cont.): Plus the flow of funds: who pays whom, when, and which entity each flow lands in.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>See the Installment Funds Flow diagram in Data Room / Product. In short: at purchase, Zed funds the merchant T+1 through Mastercard from its own balance sheet (we have no bank funding partner) and earns interchange; every flow after that is between the customer and Zed — the upfront fee and the first 1/X billing land on the enrollment-cycle statement, and each statement's installment billing converts back to revolving balance and must be paid in full by that cycle's due date under our Minimum Payment Due rules.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 1 (flow-of-funds half). Resolved 2026-09-02 by the diagram, built collaboratively with Steve; his confirmations: first 1/X bills in the enrollment cycle alongside the fee; monthly billing = 1/X + 1% add-on; single-entity issuer funded off Zed's own balance sheet, no bank partner; acquirer collapsed into the network rail; early termination as footnote only. PDF not yet uploaded to Box — SHARED-LOG row waits for Steve's confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>Revolver and pay-in-full — economics walkthrough</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Same walkthrough for a revolving balance and for a pay-in-full statement, to see how the three products differ economically.</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Interchange: as in item 1, every purchase earns Zed interchange at the swipe — payment behavior (pay in full, revolve, or installment enrollment) plays out afterwards and never changes the transaction-level economics.
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2. Do the same walkthrough for a revolving balance and for a pay-in-full statement, so we can see how the three products differ economically.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Interchange: as in 6.1, every purchase earns Zed interchange at the swipe — payment behavior (pay in full, revolve, or installment enrollment) plays out afterwards and never changes the transaction-level economics.
 Pay-in-full: charges aggregate into the statement balance at cycle end. If the cardholder pays the statement balance in full by the due date, no interest or fees are ever charged — the economics to Zed are interchange only.
 Revolving: if the cardholder pays at least the minimum payment (formula per our response to 1.2) but less than the full statement balance, the unpaid remainder revolves and accrues interest at 3% per month. Only charges made after the revolving launch are eligible to revolve.
 Missed payment: if the minimum payment is not met by the due date, late fees are charged, the account becomes past due, and a hard card freeze applies at DPD 1 (per our response to 1.4).
 Flow of funds: the purchase-side flow (merchant settlement, interchange, Zed funding from its own balance sheet) is identical for all three behaviors — see the Installment Funds Flow diagram in Data Room / Product, Part 1. For revolvers and pay-in-full, everything after settlement is simply the customer paying Zed against the monthly statement.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Fund email 2026-08-26, item 2. Flow-of-funds placeholder resolved 2026-09-02 via the same diagram as item 1. Rates grounded in 1.2 (sent). Same flow-of-funds gap as item 1. Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>"Installment fees" field definition</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>To be provided.</t>
-        </is>
-      </c>
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification pending — see METHODS.md.</t>
+          <t>Fund email 2026-08-26, bullet 2. Flow-of-funds gap resolved 2026-09-02 via the same diagram as 6.2. Rates grounded in 1.2 (sent). Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fee schedule confirmation</t>
+          <t>"Installment fees" field definition</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Drafted</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Confirm the fee schedule: add-on rate by tenor, and the origination fee formula (told 0.5% × number of months; 3% on a 6-month term). Is the fee netted from the disbursement or financed into the balance? Refundable on prepayment? Is unearned add-on interest rebated?</t>
+          <t>3. Define what the "installment fees" field in the tape contains: the upfront origination fee, the monthly add-on interest, or both combined.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors. There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement. If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
+          <t>To be provided.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
+          <t>Fund email 2026-08-26, bullet 3. Do not draft from inference — the answer depends on how the tape extract was built. Verify empirically (trace plans from the installment tape into their statement-tape rows, and/or against the warehouse) or confirm with whoever built the extract (Josif?), then write the definition. Verification pending — see METHODS.md.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Revenue fields absent from the tape</t>
+          <t>Fee schedule — rates and formula</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>The tape shows late fees and installment fees but no interchange, annual fee, upfront fee, cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
+          <t>4. Confirm the fee schedule: add-on rate by tenor, and the origination fee formula. We have been told 0.5% × number of months (3% on a 6-month term). Confirm or correct.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
+          <t>Confirmed. The origination fee is 0.5% × term months (1.5% for 3-month, 3% for 6-month, 6% for 12-month terms) and the add-on rate is 1% of original principal per month, flat across tenors.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 5. Ties to item 3 — answer both together once the extract's contents are confirmed.</t>
+          <t>Fund email 2026-08-26, bullet 4. Verified against all 4,974 plans in `Installment Tape_20260814.xlsx` (see METHODS.md): upfront/principal exactly 0.5% × months; monthly interest/principal exactly 1.0% on 4,897 plans; 77 plans show 0% interest — [Steve: promo plans? worth knowing before the fund asks]. Consistent with the 2.1 response already sent.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as % of GMV</t>
+          <t>Fee schedule — netted vs financed</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Net interchange as a percentage of GMV for the last six months, split domestic vs international if possible.</t>
+          <t>4 (cont.): Is the fee netted from the disbursement or financed into the balance?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>To be provided.</t>
+          <t>There is no cash disbursement — an installment plan converts an existing card purchase — so nothing is netted: the origination fee is charged to the account and billed on the statement.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
+          <t>Fund email 2026-08-26, bullet 4. See 9.1's verification note.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BSP rate ceilings and pricing headroom</t>
+          <t>Fee schedule — prepayment refund and interest rebate</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Both the revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom, and what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
+          <t>4 (cont.): Is it refundable on prepayment, and is unearned add-on interest rebated?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>[partial draft:] Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings. [Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
+          <t>If a plan is terminated in the first month, the origination fee is reversed and no cancellation fee applies; after the first month, the origination fee is retained and a cancellation fee equal to the current month's interest is charged. Add-on interest is billed monthly only while the plan is active, so unearned interest for remaining months is never charged (no rebate needed).</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 7. Rates verified (1.2 as sent; installment tape per METHODS.md); on the 8/12 call we already told them "all at regulatory maximums" (3%/mo ≈ 36.5% APR), so "confirmed" is consistent. The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
+          <t>Fund email 2026-08-26, bullet 4. Cancellation mechanics per Steve's 6.1 walkthrough; consistent with the funds-flow diagram footnote.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Loss figure basis, charge-off policy, restructures</t>
+          <t>Revenue fields absent from the tape</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -754,25 +753,229 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator? Charge-off policy in DPD, any change since launch, and approach to restructures/re-aging.</t>
+          <t>5. The tape shows late fees and installment fees but no interchange, no annual fee, no upfront fee, no cash advance fee, etc. Is that because those revenues do not attach to the receivable, or because they were excluded from the extract?</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume — not an annualized NCL rate. We manage to a 1–3% target range and are currently at ~2%, in line with US prime credit card benchmarks. [Steve/Claude: confirm the exact DPD threshold and computation against the warehouse before sending.] On policy: per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch. Re-aging to Current requires all arrears cleared. [Steve: whether any restructure program exists.]</t>
+          <t>[partial draft:] Interchange is earned on the merchant/network side of each transaction and never posts to the cardholder account, so it does not appear in a receivables tape. [Steve: confirm which of the other fee types exist at all as Zed products (annual fee? cash advance?) — the honest answer may simply be that these products don't exist — and whether anything that does bill to cardholders was excluded from the extract.]</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, item 8. Basis grounded in the 8/12 call notes ("dollars originated that go past due; target 1–3%, currently ~2%, in line with US prime benchmarks") — the fund heard this live, so the written answer must match it. The exact computation (DPD threshold, as-of date, cumulative vs cohort) is not specified in the notes; verify in BigQuery and record in METHODS.md before approving. Distinct from the unit econ provision line (~49% of gross revenue per active account) — if the fund juxtaposes the two, the reconciliation is originated-volume denominator vs revenue denominator.</t>
+          <t>Fund email 2026-08-26, bullet 5. Ties to 8 — answer both together once the extract's contents are confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Net interchange as % of GMV</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>6. What is your net interchange as a percentage of GMV for the last six months (if possible, split domestic vs international)?</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>To be provided.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 6. Candidate BigQuery pull — needs Steve's sign-off on definitions before running (net of network + processor costs? which GMV base? is the domestic/international split available in our data?). Unit econ file shows interchange only bundled with installment interest and fees ($6.41/account/mo), so this is a new cut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>BSP ceilings — headroom confirmation</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>7. Both your revolving rate (3%/month) and installment add-on (1%/month) sit exactly at the BSP ceilings. Confirm there is no pricing headroom.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed — our revolving rate is 3% per month and the installment add-on is 1% per month, at the current BSP ceilings.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 7 (confirmation half). Rates verified (1.2 as sent; installment tape per METHODS.md); on the 8/12 call we already told them "all at regulatory maximums" (3%/mo ≈ 36.5% APR), so "confirmed" is consistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>BSP ceilings — cut sensitivity</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>7 (cont.): …and tell us what happens to program economics if BSP cuts the ceiling at a semiannual review.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>[Steve: the sensitivity answer — impact on program economics of a ceiling cut, and any mitigants (fee mix, funding cost, underwriting).]</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 7 (sensitivity half). The headroom/sensitivity narrative is strategy — Steve's voice required. Consider whether the unit econ pro forma should be the quantitative backbone of the answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Loss figure — basis and denominator</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>8. What's the basis for the ~2% loss figure provided (30+/90+ DPD, annualized NCL, cumulative) and its denominator?</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>The ~2% figure is our headline default metric as discussed on our call: dollars originated that go past due, i.e. past-due originated volume over cumulative originated volume — not an annualized NCL rate. We manage to a 1–3% target range and are currently at ~2%, in line with US prime credit card benchmarks. [Steve/Claude: confirm the exact DPD threshold and computation against the warehouse before sending.]</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 8 (basis half). Grounded in the 8/12 call notes ("dollars originated that go past due; target 1–3%, currently ~2%, in line with US prime benchmarks") — the fund heard this live, so the written answer must match it. The exact computation (DPD threshold, as-of date, cumulative vs cohort) is not specified in the notes; verify in BigQuery and record in METHODS.md before approving. Distinct from the unit econ provision line (~49% of gross revenue per active account) — if the fund juxtaposes the two, the reconciliation is originated-volume denominator vs revenue denominator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Charge-off policy and changes since launch</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>8 (cont.): We'd also appreciate your charge-off policy in DPD, and any change to it since launch.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Per our ECL policy we provision 100% at 180+ DPD; we have not yet formally written off balances while we stand up the collections-substantiation and BIR documentation required, and the policy is unchanged since launch.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 8 (policy half). Drafted 2026-09-01 from the 8/12 call context; review wording with Steve before approving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Restructures and re-aging</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>8 (cont.): …and your approach to restructures/re-aging.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Re-aging to Current requires all arrears cleared. [Steve: whether any restructure program exists.]</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Fund email 2026-08-26, bullet 8 (restructures half). Restructure-program existence is unconfirmed — do not answer without Steve.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Claude: revise (see notes),Discuss"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Rewrite item 7: pay-in-full is a behavior not a SKU; full revolving explainer (v10)
- Leads with the premise correction: charge card deprecated (5/25 launch,
  6/1 first MPD statements, 6/15 final cohort transition, 100% on revolving)
- First-principles revolving mechanics from the internal CS support guide:
  grace period loss/regain, 0.1%/day adjusted-daily-balance interest from
  statement cut-off, residual interest, Php1,000 late penalty, installment interaction
- Internal note flags: late penalty never sent before; assessment timing pending
  internally (omitted); supersedes 1.2's eligible-to-revolve line consistently

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -584,18 +584,25 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Interchange: as in 6.1, every purchase earns Zed interchange at the swipe — payment behavior (pay in full, revolve, or installment enrollment) plays out afterwards and never changes the transaction-level economics.
-Pay-in-full: charges aggregate into the statement balance at cycle end. If the cardholder pays the statement balance in full by the due date, no interest or fees are ever charged — the economics to Zed are interchange only.
-Revolving: if the cardholder pays at least the minimum payment (formula per our response to 1.2) but less than the full statement balance, the unpaid remainder revolves and accrues interest at 3% per month. Only charges made after the revolving launch are eligible to revolve.
-Missed payment: if the minimum payment is not met by the due date, late fees are charged, the account becomes past due, and a hard card freeze applies at DPD 1 (per our response to 1.4).
-Flow of funds: the purchase-side flow (merchant settlement, interchange, Zed funding from its own balance sheet) is identical for all three behaviors — see the Installment Funds Flow diagram in Data Room / Product, Part 1. For revolvers and pay-in-full, everything after settlement is simply the customer paying Zed against the monthly statement.</t>
+          <t>One clarification on the premise first: "pay in full" is not a separate product — it refers to the charge-card dynamic we have since deprecated. We launched revolving on May 25th. The first statements carrying a Minimum Payment Due below the statement ending balance were generated June 1; the second and final cohort of users still on the charge-card behavior (where MPD = statement ending balance) was transitioned on June 15. Since then, 100% of the customer base is on the revolving product. Cardholders can always opt to pay their balance in full — like any credit card — to avoid interest, but it is no longer required. So there is one card product (a revolving credit card with an installment feature), and paying in full vs. revolving are payment behaviors on that product, not separate SKUs for different customer subsets.
+Interchange: as in 6.1, every purchase earns Zed interchange at the swipe — payment behavior plays out afterwards and never changes the transaction-level economics.
+How revolving works, from first principles:
+Statement cycle: purchases post to the balance through the cycle; at cycle close we generate a statement fixing the statement balance, the Minimum Payment Due (formula per our response to 1.2 — in short, 100% of billed installment amounts, late fees and past-due amounts, plus 10% of the remaining statement balance, floored at ₱1,000), and the payment due date.
+Grace period — the pay-in-full behavior: if the cardholder paid the prior statement in full, no interest accrues on purchases through the due date. A cardholder who pays the statement balance in full by the due date every cycle never pays interest; Zed's economics on these users are interchange only.
+Losing the grace period: paying anything less than the full statement balance by the due date — even well above the MPD — ends the grace period. From that point interest accrues daily on the unpaid balance starting from the statement cut-off date (day 1 of interest is the statement day itself), and the accrued interest is billed on the next statement.
+How interest is computed: 3% per month, accrued daily at 0.1%/day on the adjusted daily balance (we use the 30-day banking standard for the daily rate, so a 31-day month accrues 3.1% and a 28-day month 2.8%). Payments reduce the accruing balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance; they pay ₱250 on day 11 and nothing else; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
+Residual interest: once the grace period is lost, paying the balance in full mid-cycle stops accrual going forward, but the interest already accrued for the days the balance existed still bills on the following statement.
+Regaining the grace period: pay the total balance in full by the payment due date; the grace period resumes from the following billing cycle.
+Missed payment: if the MPD is not met by the due date, a ₱1,000 late payment penalty applies, the account is past due, and a hard card freeze applies at DPD 1 (per our response to 1.4). Interest continues to accrue on the unpaid balance while delinquent, and the past-due amount includes accrued finance charges.
+Installment interaction, for completeness: billed installment amounts accrue no interest for cardholders whose grace period is intact; once the grace period is lost, they accrue daily interest from the statement date until paid — consistent with the billed-installment-converts-to-revolving mechanics in 6.1/6.2.
+Flow of funds: the purchase-side flow (merchant settlement, interchange, Zed funding from its own balance sheet) is identical for all payment behaviors — see the Installment Funds Flow diagram in Data Room / Product, Part 1. For revolvers and full payers, everything after settlement is simply the customer paying Zed against the monthly statement.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, bullet 2. Flow-of-funds gap resolved 2026-09-02 via the same diagram as 6.2. Rates grounded in 1.2 (sent). Context the fund heard on the 8/12 call: revolving is the primary revenue driver; 33% of users use installments or revolving, 7% both, 10% installments only; installment users skew transactor. Verify these figures before putting them in a written response.</t>
+          <t>Fund email 2026-08-26, bullet 2. Rewritten 2026-09-02 per Steve: FPF appeared to assume pay-in-full is a separate SKU — the correction (charge card deprecated; June 1 / June 15 transition; 100% on revolving) leads the answer and matches 1.1 as sent. Revolving mechanics sourced from the internal "Revolving Credit Card Support Guide" (Notion / Customer Success, last edited 2026-08-13): grace-period loss/regain, daily 0.1% adjusted-daily-balance accrual from statement cut-off, residual interest, ₱1,000 late payment penalty. Flags: (a) the ₱1,000 late penalty was not in any sent response and is distinct from 1.2's ₱1,000 MPD floor — don't conflate; (b) guide says penalty assessment timing (DPD) is still pending internally, so the answer deliberately omits it; (c) 1.2-sent line "only charges after revolving launched were able to revolve" is superseded by the fuller transition narrative — consistent, since pre-transition statements required full payment. Call-context figures (33%/7%/10% mix) still unverified — keep out of written responses. Flow-of-funds gap resolved via the same diagram as 6.2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Item 7: late fee bills after 2-day grace past due date, per i2c config (v11)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -593,7 +593,7 @@
 How interest is computed: 3% per month, accrued daily at 0.1%/day on the adjusted daily balance (we use the 30-day banking standard for the daily rate, so a 31-day month accrues 3.1% and a 28-day month 2.8%). Payments reduce the accruing balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance; they pay ₱250 on day 11 and nothing else; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
 Residual interest: once the grace period is lost, paying the balance in full mid-cycle stops accrual going forward, but the interest already accrued for the days the balance existed still bills on the following statement.
 Regaining the grace period: pay the total balance in full by the payment due date; the grace period resumes from the following billing cycle.
-Missed payment: if the MPD is not met by the due date, a ₱1,000 late payment penalty applies, the account is past due, and a hard card freeze applies at DPD 1 (per our response to 1.4). Interest continues to accrue on the unpaid balance while delinquent, and the past-due amount includes accrued finance charges.
+Missed payment: if the MPD is not met by the due date, the account is past due and a hard card freeze applies at DPD 1 (per our response to 1.4). A ₱1,000 late payment penalty is charged if payment still has not been made within the 2-day late-payment grace period following the due date. Interest continues to accrue on the unpaid balance while delinquent, and the past-due amount includes accrued finance charges.
 Installment interaction, for completeness: billed installment amounts accrue no interest for cardholders whose grace period is intact; once the grace period is lost, they accrue daily interest from the statement date until paid — consistent with the billed-installment-converts-to-revolving mechanics in 6.1/6.2.
 Flow of funds: the purchase-side flow (merchant settlement, interchange, Zed funding from its own balance sheet) is identical for all payment behaviors — see the Installment Funds Flow diagram in Data Room / Product, Part 1. For revolvers and full payers, everything after settlement is simply the customer paying Zed against the monthly statement.</t>
         </is>
@@ -602,7 +602,7 @@
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fund email 2026-08-26, bullet 2. Rewritten 2026-09-02 per Steve: FPF appeared to assume pay-in-full is a separate SKU — the correction (charge card deprecated; June 1 / June 15 transition; 100% on revolving) leads the answer and matches 1.1 as sent. Revolving mechanics sourced from the internal "Revolving Credit Card Support Guide" (Notion / Customer Success, last edited 2026-08-13): grace-period loss/regain, daily 0.1% adjusted-daily-balance accrual from statement cut-off, residual interest, ₱1,000 late payment penalty. Flags: (a) the ₱1,000 late penalty was not in any sent response and is distinct from 1.2's ₱1,000 MPD floor — don't conflate; (b) guide says penalty assessment timing (DPD) is still pending internally, so the answer deliberately omits it; (c) 1.2-sent line "only charges after revolving launched were able to revolve" is superseded by the fuller transition narrative — consistent, since pre-transition statements required full payment. Call-context figures (33%/7%/10% mix) still unverified — keep out of written responses. Flow-of-funds gap resolved via the same diagram as 6.2.</t>
+          <t>Fund email 2026-08-26, bullet 2. Rewritten 2026-09-02 per Steve: FPF appeared to assume pay-in-full is a separate SKU — the correction (charge card deprecated; June 1 / June 15 transition; 100% on revolving) leads the answer and matches 1.1 as sent. Revolving mechanics sourced from the internal "Revolving Credit Card Support Guide" (Notion / Customer Success, last edited 2026-08-13): grace-period loss/regain, daily 0.1% adjusted-daily-balance accrual from statement cut-off, residual interest, ₱1,000 late payment penalty. Flags: (a) the ₱1,000 late penalty was not in any sent response and is distinct from 1.2's ₱1,000 MPD floor — don't conflate; (b) penalty timing confirmed 2026-09-02 from the i2c program config (Zed_Card_NNB, Credit Card Rules → Statement, screenshot from Steve): Late Payment Grace Period = 2 days after the due date — resolves the guide's "timing pending"; the i2c Delinquency Grace Period field appears unset, consistent with freeze at DPD 1; (c) 1.2-sent line "only charges after revolving launched were able to revolve" is superseded by the fuller transition narrative — consistent, since pre-transition statements required full payment. Call-context figures (33%/7%/10% mix) still unverified — keep out of written responses. Flow-of-funds gap resolved via the same diagram as 6.2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Item 7: plain-language interest mechanics; retroactive-to-statement-day nuance (v15)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191mfdzKjQFrnE6DWH5jJQc
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -589,8 +589,10 @@
 How revolving works, from first principles:
 Statement cycle: purchases post to the balance through the cycle; at cycle close we generate a statement fixing the statement balance, the Minimum Payment Due (formula per our response to 1.2 — in short, 100% of billed installment amounts, late fees and past-due amounts, plus 10% of the remaining statement balance, floored at ₱1,000), and the payment due date.
 Grace period — the pay-in-full behavior: if the cardholder paid the prior statement in full, no interest accrues on purchases through the due date. A cardholder who pays the statement balance in full by the due date every cycle never pays interest; Zed's economics on these users are interchange only.
-Losing the grace period: paying anything less than the full statement balance by the due date — even well above the MPD — ends the grace period. From that point interest accrues daily on the unpaid balance starting from the statement cut-off date (day 1 of interest is the statement day itself), and the accrued interest is billed on the next statement.
-How interest is computed: 3% per month, accrued daily at 0.1%/day on the adjusted daily balance (we use the 30-day banking standard for the daily rate, so a 31-day month accrues 3.1% and a 28-day month 2.8%). Payments reduce the accruing balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance; they pay ₱250 on day 11 and nothing else; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
+Losing the grace period: paying anything less than the full statement balance by the due date — even well above the MPD — loses the grace period.
+What interest is charged on: only balances that have been billed on a statement. Purchases made during the current cycle have not been billed yet, so they accrue no interest while the cycle is running — they become interest-bearing only once they appear on a statement that then isn't paid in full.
+When interest starts: on the statement day, not the due date. For a cardholder who has already lost their grace period, each statement's unpaid balance starts accruing daily interest from the day the statement is generated. Just as important: in the very cycle where the grace period is lost, interest is applied back to the last statement day — a cardholder who pays less than the full balance at the due date is charged daily interest counted from the day that statement was generated, not from the day they underpaid.
+How the daily math works: 3% per month is applied as 0.1% per day (30-day banking standard, so a 31-day month accrues 3.1% and a 28-day month 2.8%) on each day's outstanding billed balance, and payments reduce that balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance and pays ₱250 on day 11; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
 Residual interest: once the grace period is lost, paying the balance in full mid-cycle stops accrual going forward, but the interest already accrued for the days the balance existed still bills on the following statement.
 Regaining the grace period: pay the total balance in full by the payment due date; the grace period resumes from the following billing cycle.
 Missed payment: if the MPD is not met by the due date, the account is past due and a hard card freeze applies at DPD 1 (per our response to 1.4). A ₱1,000 late payment penalty is charged if payment still has not been made within the 2-day late-payment grace period following the due date. Interest continues to accrue on the unpaid balance while delinquent, and the past-due amount includes accrued finance charges.

</xml_diff>

<commit_message>
Revert "Item 7: plain-language interest mechanics; retroactive-to-statement-day nuance (v15)"
This reverts commit cfd270e873d2a4e6c7fc8f59220434cd524b4214.
</commit_message>
<xml_diff>
--- a/WORKING - Diligence Responses.xlsx
+++ b/WORKING - Diligence Responses.xlsx
@@ -589,10 +589,8 @@
 How revolving works, from first principles:
 Statement cycle: purchases post to the balance through the cycle; at cycle close we generate a statement fixing the statement balance, the Minimum Payment Due (formula per our response to 1.2 — in short, 100% of billed installment amounts, late fees and past-due amounts, plus 10% of the remaining statement balance, floored at ₱1,000), and the payment due date.
 Grace period — the pay-in-full behavior: if the cardholder paid the prior statement in full, no interest accrues on purchases through the due date. A cardholder who pays the statement balance in full by the due date every cycle never pays interest; Zed's economics on these users are interchange only.
-Losing the grace period: paying anything less than the full statement balance by the due date — even well above the MPD — loses the grace period.
-What interest is charged on: only balances that have been billed on a statement. Purchases made during the current cycle have not been billed yet, so they accrue no interest while the cycle is running — they become interest-bearing only once they appear on a statement that then isn't paid in full.
-When interest starts: on the statement day, not the due date. For a cardholder who has already lost their grace period, each statement's unpaid balance starts accruing daily interest from the day the statement is generated. Just as important: in the very cycle where the grace period is lost, interest is applied back to the last statement day — a cardholder who pays less than the full balance at the due date is charged daily interest counted from the day that statement was generated, not from the day they underpaid.
-How the daily math works: 3% per month is applied as 0.1% per day (30-day banking standard, so a 31-day month accrues 3.1% and a 28-day month 2.8%) on each day's outstanding billed balance, and payments reduce that balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance and pays ₱250 on day 11; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
+Losing the grace period: paying anything less than the full statement balance by the due date — even well above the MPD — ends the grace period. From that point interest accrues daily on the unpaid balance starting from the statement cut-off date (day 1 of interest is the statement day itself), and the accrued interest is billed on the next statement.
+How interest is computed: 3% per month, accrued daily at 0.1%/day on the adjusted daily balance (we use the 30-day banking standard for the daily rate, so a 31-day month accrues 3.1% and a 28-day month 2.8%). Payments reduce the accruing balance the day they post. Example: a cardholder who has lost their grace period carries a ₱1,000 statement balance; they pay ₱250 on day 11 and nothing else; interest accrues on ₱1,000 for days 1–10 and on ₱750 for days 11–30, and the summed daily interest is billed on the next statement.
 Residual interest: once the grace period is lost, paying the balance in full mid-cycle stops accrual going forward, but the interest already accrued for the days the balance existed still bills on the following statement.
 Regaining the grace period: pay the total balance in full by the payment due date; the grace period resumes from the following billing cycle.
 Missed payment: if the MPD is not met by the due date, the account is past due and a hard card freeze applies at DPD 1 (per our response to 1.4). A ₱1,000 late payment penalty is charged if payment still has not been made within the 2-day late-payment grace period following the due date. Interest continues to accrue on the unpaid balance while delinquent, and the past-due amount includes accrued finance charges.

</xml_diff>